<commit_message>
feat: lógica de meses para validThrough e limpeza de salários
</commit_message>
<xml_diff>
--- a/modelo_importacao_vagas.xlsx
+++ b/modelo_importacao_vagas.xlsx
@@ -543,8 +543,8 @@
       <c r="M3">
         <v>900</v>
       </c>
-      <c r="N3" t="str">
-        <v>2024-12-31</v>
+      <c r="N3">
+        <v>3</v>
       </c>
     </row>
     <row r="4">
@@ -587,8 +587,8 @@
       <c r="M4">
         <v>1200</v>
       </c>
-      <c r="N4" t="str">
-        <v>2024-12-31</v>
+      <c r="N4">
+        <v>6</v>
       </c>
     </row>
     <row r="5">
@@ -631,8 +631,8 @@
       <c r="M5">
         <v>1000</v>
       </c>
-      <c r="N5" t="str">
-        <v>2024-12-31</v>
+      <c r="N5">
+        <v>12</v>
       </c>
     </row>
   </sheetData>

</xml_diff>